<commit_message>
Hoan thanh bai tap b4
</commit_message>
<xml_diff>
--- a/Template/DSSV.xlsx
+++ b/Template/DSSV.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\xayda\source\repos\CSharpLearning\Template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B75685D-4957-40C3-BABD-712F08C748F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D94B6B4-8C1F-4225-AE05-EF8A45B745B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1950" yWindow="1950" windowWidth="15375" windowHeight="7785" xr2:uid="{341E9F9D-FEB9-46B6-AA58-3C6D59801EF6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{341E9F9D-FEB9-46B6-AA58-3C6D59801EF6}"/>
   </bookViews>
   <sheets>
     <sheet name="DSSV" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Mã Sinh Viên</t>
   </si>
@@ -58,6 +58,12 @@
   </si>
   <si>
     <t>Phạm Văn Dương</t>
+  </si>
+  <si>
+    <t>Ngày sinh</t>
+  </si>
+  <si>
+    <t>28/11/2007</t>
   </si>
 </sst>
 </file>
@@ -107,12 +113,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -429,16 +438,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60B79B58-A1B7-41A6-B780-D03715268E18}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.5703125" customWidth="1"/>
     <col min="2" max="2" width="22.85546875" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="5" width="18.140625" customWidth="1"/>
+    <col min="4" max="4" width="15.5703125" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="18.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -449,13 +459,16 @@
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -465,14 +478,17 @@
       <c r="C2" s="1">
         <v>22</v>
       </c>
-      <c r="D2" s="1">
+      <c r="D2" s="3">
+        <v>38176</v>
+      </c>
+      <c r="E2" s="1">
         <v>8.6999999999999993</v>
       </c>
-      <c r="E2" s="1">
+      <c r="F2" s="1">
         <v>7.5</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -482,14 +498,17 @@
       <c r="C3" s="1">
         <v>20</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D3" s="3">
+        <v>39057</v>
+      </c>
+      <c r="E3" s="1">
         <v>9.8000000000000007</v>
       </c>
-      <c r="E3" s="1">
+      <c r="F3" s="1">
         <v>8.1999999999999993</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -499,14 +518,17 @@
       <c r="C4" s="1">
         <v>19</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="1">
         <v>9.5</v>
       </c>
-      <c r="E4" s="1">
+      <c r="F4" s="1">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -516,14 +538,17 @@
       <c r="C5" s="1">
         <v>15</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5" s="3">
+        <v>41192</v>
+      </c>
+      <c r="E5" s="1">
         <v>7.5</v>
       </c>
-      <c r="E5" s="1">
+      <c r="F5" s="1">
         <v>7.1</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -533,14 +558,17 @@
       <c r="C6" s="1">
         <v>18</v>
       </c>
-      <c r="D6" s="1">
+      <c r="D6" s="3">
+        <v>40247</v>
+      </c>
+      <c r="E6" s="1">
         <v>7</v>
       </c>
-      <c r="E6" s="1">
+      <c r="F6" s="1">
         <v>7.6</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -550,10 +578,11 @@
       <c r="C7" s="1">
         <v>20</v>
       </c>
-      <c r="D7" s="1">
+      <c r="D7" s="1"/>
+      <c r="E7" s="1">
         <v>9</v>
       </c>
-      <c r="E7" s="1">
+      <c r="F7" s="1">
         <v>8</v>
       </c>
     </row>

</xml_diff>